<commit_message>
feat(presupuesto): anadir serie Efapel MEC 21 + Apolo 5000 y modo seleccion racional mas economica
</commit_message>
<xml_diff>
--- a/base_datos_precio_oficial.xlsx
+++ b/base_datos_precio_oficial.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M350"/>
+  <dimension ref="A1:M375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21772,6 +21772,1531 @@
         </is>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>ART-0350</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>EFA-21011</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Mecanismo Interruptor Unipolar 10AX 250V Efapel MEC 21 (Ref. 21011)</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J351" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="K351" t="n">
+        <v>21</v>
+      </c>
+      <c r="L351" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>Mecanismo universal para vestir con Tecla Serie Apolo 5000 / Logus 90</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>ART-0351</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>EFA-21071</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>Mecanismo Conmutador 10AX 250V Efapel MEC 21 (Ref. 21071)</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J352" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="K352" t="n">
+        <v>21</v>
+      </c>
+      <c r="L352" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>Mecanismo conmutador universal para vestir con Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>ART-0352</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>EFA-21051</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>Mecanismo Cruzamiento 10AX 250V Efapel MEC 21 (Ref. 21051)</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J353" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="K353" t="n">
+        <v>21</v>
+      </c>
+      <c r="L353" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>Mecanismo cruzamiento universal Efapel MEC 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>ART-0353</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>EFA-21151</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>Mecanismo Pulsador 10A 250V Efapel MEC 21 (Ref. 21151)</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J354" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="K354" t="n">
+        <v>21</v>
+      </c>
+      <c r="L354" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>Mecanismo pulsador para timbre o telerruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>ART-0354</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>EFA-21021</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>Mecanismo Doble Interruptor 10AX Efapel MEC 21 (Ref. 21021)</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J355" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K355" t="n">
+        <v>21</v>
+      </c>
+      <c r="L355" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>Mecanismo doble interruptor 2 circuitos</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>ART-0355</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>EFA-21031</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>Mecanismo Doble Conmutador 10AX Efapel MEC 21 (Ref. 21031)</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J356" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="K356" t="n">
+        <v>21</v>
+      </c>
+      <c r="L356" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>Mecanismo doble conmutador para 2 puntos conmutados</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>ART-0356</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>EFA-21111</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>Base de Enchufe Schuko 16A 250V 2P+T con Obturador Efapel MEC 21 (Ref. 21111)</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J357" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="K357" t="n">
+        <v>21</v>
+      </c>
+      <c r="L357" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>Base schuko con seguridad infantil para vestir con Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>ART-0357</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>EFA-21381</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>Mecanismo Toma RJ45 Cat 6 UTP Datos Efapel MEC 21 (Ref. 21381)</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J358" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K358" t="n">
+        <v>21</v>
+      </c>
+      <c r="L358" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>Toma de red informática Cat 6 conector Keystone</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>ART-0358</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>EFA-21541</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>Mecanismo Toma TV-R / SAT Final Efapel MEC 21 (Ref. 21541)</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J359" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K359" t="n">
+        <v>21</v>
+      </c>
+      <c r="L359" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>Toma televisión y radio satélite final</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>ART-0359</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>EFA-21281</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>Mecanismo Pulsador Persianas Subir/Bajar Efapel MEC 21 (Ref. 21281)</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J360" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="K360" t="n">
+        <v>21</v>
+      </c>
+      <c r="L360" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>Mando motor persianas con enclavamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>ART-0360</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>EFA-50910-TBR</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>Tecla Simple para Interruptor/Conmutador Efapel Apolo 5000 Blanco (Ref. 50910 TBR)</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J361" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="K361" t="n">
+        <v>21</v>
+      </c>
+      <c r="L361" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>Tecla embellecedora blanca para mecanismo MEC 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>ART-0361</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>EFA-50912-TBR</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>Tecla Doble para Mecanismo Doble Efapel Apolo 5000 Blanco (Ref. 50912 TBR)</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J362" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K362" t="n">
+        <v>21</v>
+      </c>
+      <c r="L362" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>Tecla partida doble para MEC 21 doble</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>ART-0362</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>EFA-50918-TBR</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>Tecla Persianas con Flechas Efapel Apolo 5000 Blanco (Ref. 50918 TBR)</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J363" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K363" t="n">
+        <v>21</v>
+      </c>
+      <c r="L363" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>Tecla serigrafiada para persianas motorizadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>ART-0363</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>EFA-50942-TBR</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>Frontal Tapa Toma RJ45 Efapel Apolo 5000 Blanco (Ref. 50942 TBR)</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J364" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K364" t="n">
+        <v>21</v>
+      </c>
+      <c r="L364" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>Frontal embellecedor para conector RJ45</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>ART-0364</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>EFA-50951-TBR</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>Frontal Tapa Toma TV-R Efapel Apolo 5000 Blanco (Ref. 50951 TBR)</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J365" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K365" t="n">
+        <v>21</v>
+      </c>
+      <c r="L365" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>Frontal embellecedor para toma antena TV-R</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>ART-0365</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Marcos / Placas</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>EFA-50920-TBR</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>Marco 1 Elemento Efapel Apolo 5000 Blanco (Ref. 50920 TBR)</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J366" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="K366" t="n">
+        <v>21</v>
+      </c>
+      <c r="L366" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>Marco embellecedor simple serie económica Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>ART-0366</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Marcos / Placas</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>EFA-50922-TBR</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>Marco 2 Elementos Efapel Apolo 5000 Blanco (Ref. 50922 TBR)</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J367" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K367" t="n">
+        <v>21</v>
+      </c>
+      <c r="L367" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>Marco doble horizontal/vertical Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>ART-0367</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Marcos / Placas</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>EFA-50923-TBR</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>Marco 3 Elementos Efapel Apolo 5000 Blanco (Ref. 50923 TBR)</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J368" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="K368" t="n">
+        <v>21</v>
+      </c>
+      <c r="L368" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>Marco triple horizontal/vertical Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>ART-0368</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Marcos / Placas</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>EFA-50924-TBR</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>Marco 4 Elementos Efapel Apolo 5000 Blanco (Ref. 50924 TBR)</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J369" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="K369" t="n">
+        <v>21</v>
+      </c>
+      <c r="L369" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>Marco cuádruple horizontal/vertical Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>ART-0369</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>EFA-KIT-INT-5000</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>Conjunto Interruptor Unipolar Efapel MEC 21 + Tecla/Marco Apolo 5000 Blanco (Ref. 21011+50910+50920)</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J370" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="K370" t="n">
+        <v>21</v>
+      </c>
+      <c r="L370" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>Conjunto completo listo para instalar (mecanismo + tecla + marco)</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>ART-0370</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>EFA-KIT-CONM-5000</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>Conjunto Conmutador Efapel MEC 21 + Tecla/Marco Apolo 5000 Blanco (Ref. 21071+50910+50920)</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J371" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="K371" t="n">
+        <v>21</v>
+      </c>
+      <c r="L371" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>Conjunto completo conmutador + tecla + marco</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>ART-0371</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>EFA-KIT-CRUZ-5000</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>Conjunto Cruzamiento Efapel MEC 21 + Tecla/Marco Apolo 5000 Blanco (Ref. 21051+50910+50920)</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J372" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="K372" t="n">
+        <v>21</v>
+      </c>
+      <c r="L372" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>Conjunto completo cruzamiento + tecla + marco</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>ART-0372</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>EFA-KIT-PULS-5000</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>Conjunto Pulsador Efapel MEC 21 + Tecla/Marco Apolo 5000 Blanco (Ref. 21151+50910+50920)</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J373" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="K373" t="n">
+        <v>21</v>
+      </c>
+      <c r="L373" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>Conjunto completo pulsador + tecla + marco</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>ART-0373</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>EFA-KIT-SCH-5000</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>Conjunto Base Enchufe Schuko 16A 2P+T Efapel MEC 21 + Marco Apolo 5000 Blanco (Ref. 21111+50920)</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J374" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K374" t="n">
+        <v>21</v>
+      </c>
+      <c r="L374" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>Base schuko completa con marco Apolo 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>ART-0374</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>1. Gama Ultra Económica / Base</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Mecanismos</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Efapel</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>MEC 21 / Apolo 5000</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>EFA-KIT-RJ45-5000</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>Conjunto Toma RJ45 Cat 6 Efapel MEC 21 + Frontal/Marco Apolo 5000 Blanco (Ref. 21381+50942+50920)</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J375" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="K375" t="n">
+        <v>21</v>
+      </c>
+      <c r="L375" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>Toma de datos Cat 6 completa con frontal y marco</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(cuadro): corregir seleccion de envolvente de cuadro electrico DIN y cajas de registro/mecanismos
</commit_message>
<xml_diff>
--- a/base_datos_precio_oficial.xlsx
+++ b/base_datos_precio_oficial.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M375"/>
+  <dimension ref="A1:M379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23297,6 +23297,250 @@
         </is>
       </c>
     </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>ART-0375</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1. Gama Económica</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Cuadros y Envolventes</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Solera</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Arelos / Indubox</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>SOL-12MOD-EMP</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Caja de Distribución Empotrar Solera Arelos 12 Módulos DIN Puerta Blanca</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J376" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="K376" t="n">
+        <v>21</v>
+      </c>
+      <c r="L376" t="n">
+        <v>13.55</v>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>Cuadro general empotrar para electrificación básica (12 módulos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>ART-0376</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>1. Gama Económica</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Cuadros y Envolventes</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Solera</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Arelos / Indubox</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>SOL-24MOD-EMP</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Caja de Distribución Empotrar Solera Arelos 24 Módulos DIN (2 Filas) Puerta Blanca</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J377" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="K377" t="n">
+        <v>21</v>
+      </c>
+      <c r="L377" t="n">
+        <v>22.38</v>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>Cuadro general empotrar para electrificación elevada (24 módulos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>ART-0377</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>1. Gama Económica</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Cuadros y Envolventes</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Chint</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>e-Box</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>CHT-EBOX-12</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Caja de Distribución Modular Empotrar Chint e-Box 12 Módulos</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J378" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="K378" t="n">
+        <v>21</v>
+      </c>
+      <c r="L378" t="n">
+        <v>13.07</v>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>Cuadro modular para protecciones Chint 12 módulos</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>ART-0378</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>1. Gama Económica</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Cuadros y Envolventes</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Chint</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>e-Box</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Mayorista / Distribución Especializada</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>CHT-EBOX-24</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Caja de Distribución Modular Empotrar Chint e-Box 24 Módulos (2 Filas)</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="J379" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K379" t="n">
+        <v>21</v>
+      </c>
+      <c r="L379" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>Cuadro modular para protecciones Chint 24 módulos</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(materiales): permitir seleccion independiente de tecnologia de cable (H07Z1-K/H07V-K) y tecnologia de tubo (LH/PVC)
</commit_message>
<xml_diff>
--- a/base_datos_precio_oficial.xlsx
+++ b/base_datos_precio_oficial.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M379"/>
+  <dimension ref="A1:M396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23541,6 +23541,1043 @@
         </is>
       </c>
     </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>ART-0379</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Reformas</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Canalización Tubos</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC Estándar</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>OBR-TUBO-PVC-M16</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC M16 Normal / Estándar 320N (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J380" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="K380" t="n">
+        <v>21</v>
+      </c>
+      <c r="L380" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>Tubo corrugado flexible de PVC para canalizaciones empotradas ordinarias</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>ART-0380</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Reformas</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Canalización Tubos</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC Estándar</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>OBR-TUBO-PVC-M20</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC M20 Normal / Estándar 320N (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J381" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K381" t="n">
+        <v>21</v>
+      </c>
+      <c r="L381" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>Tubo corrugado flexible de PVC para circuitos de alumbrado y enchufes</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>ART-0381</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Reformas</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Canalización Tubos</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC Estándar</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>OBR-TUBO-PVC-M25</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC M25 Normal / Estándar 320N (Rollo 50m)</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J382" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="K382" t="n">
+        <v>21</v>
+      </c>
+      <c r="L382" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>Tubo corrugado flexible de PVC para circuitos de fuerza, cocina y horno</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>ART-0382</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Reformas</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Canalización Tubos</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC Estándar</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>OBR-TUBO-PVC-M32</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>Tubo Corrugado PVC M32 Normal / Estándar 320N (Rollo 25m)</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J383" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="K383" t="n">
+        <v>21</v>
+      </c>
+      <c r="L383" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>Tubo corrugado flexible de PVC para derivaciones principales y enlace</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>ART-0383</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-15-AZ</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x1.5 mm² PVC Normal Azul (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J384" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="K384" t="n">
+        <v>21</v>
+      </c>
+      <c r="L384" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC neutro azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>ART-0384</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-15-NE</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x1.5 mm² PVC Normal Negro (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J385" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="K385" t="n">
+        <v>21</v>
+      </c>
+      <c r="L385" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC fase negro</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>ART-0385</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-15-MA</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x1.5 mm² PVC Normal Marrón (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J386" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="K386" t="n">
+        <v>21</v>
+      </c>
+      <c r="L386" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC fase marrón</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>ART-0386</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-15-GR</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x1.5 mm² PVC Normal Gris (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J387" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="K387" t="n">
+        <v>21</v>
+      </c>
+      <c r="L387" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC fase gris</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>ART-0387</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-15-TT</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x1.5 mm² PVC Normal Amarillo/Verde (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J388" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="K388" t="n">
+        <v>21</v>
+      </c>
+      <c r="L388" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC toma de tierra</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>ART-0388</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-25-AZ</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x2.5 mm² PVC Normal Azul (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J389" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K389" t="n">
+        <v>21</v>
+      </c>
+      <c r="L389" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC neutro azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>ART-0389</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-25-NE</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x2.5 mm² PVC Normal Negro (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J390" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K390" t="n">
+        <v>21</v>
+      </c>
+      <c r="L390" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC fase negro</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>ART-0390</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-25-MA</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x2.5 mm² PVC Normal Marrón (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J391" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K391" t="n">
+        <v>21</v>
+      </c>
+      <c r="L391" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC fase marrón</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>ART-0391</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-25-GR</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x2.5 mm² PVC Normal Gris (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J392" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K392" t="n">
+        <v>21</v>
+      </c>
+      <c r="L392" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC fase gris</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>ART-0392</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-25-TT</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x2.5 mm² PVC Normal Amarillo/Verde (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J393" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K393" t="n">
+        <v>21</v>
+      </c>
+      <c r="L393" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC toma de tierra</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>ART-0393</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-40</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x4.0 mm² PVC Normal (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J394" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K394" t="n">
+        <v>21</v>
+      </c>
+      <c r="L394" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC para líneas C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>ART-0394</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-60</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x6.0 mm² PVC Normal (Rollo 100m)</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J395" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="K395" t="n">
+        <v>21</v>
+      </c>
+      <c r="L395" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>Conductor flexible unipolar de cobre clase 5 con aislamiento PVC para cocina/horno C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>ART-0395</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>1. Gama Estándar / Tradicional</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Conductores</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>General Cable / Top Cable</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>H07V-K (PVC)</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Obramat</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>OBR-CAB-PVC-100</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>Cable H07V-K 1x10.0 mm² PVC Normal (Corte/m)</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J396" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="K396" t="n">
+        <v>21</v>
+      </c>
+      <c r="L396" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>Conductor unipolar de cobre clase 5 para derivación y cuadro general</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>